<commit_message>
Laminas comunales de Educacion regeneradas
Lote 1 de 6.
El commit original (b1bed81b) cambiaba 13.973 archivos y 2,40 GB de objetos
nuevos en una sola pieza. GitHub rechaza los push sobre 2 GB por HTTPS, y SSH
esta bloqueado en esta red, asi que ese commit no podia subir nunca: el HTTP 500
no era un error transitorio sino el limite. Se trocea por dimension, que es un
corte con sentido, no alfabetico.
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_e_basbrut_a_2018_aysen.xlsx
+++ b/output/graficos_dimensiones/comunal_e_basbrut_a_2018_aysen.xlsx
@@ -54,12 +54,12 @@
     <t xml:space="preserve">Río Ibáñez</t>
   </si>
   <si>
+    <t xml:space="preserve">O'Higgins</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tortel</t>
   </si>
   <si>
-    <t xml:space="preserve">O'Higgins</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cochrane</t>
   </si>
   <si>
@@ -72,7 +72,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-06 21:19</t>
+    <t xml:space="preserve">2026-09-10 00:24</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -621,7 +621,7 @@
         <v>12</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>11303</v>
+        <v>11302</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>2018</v>
@@ -638,7 +638,7 @@
         <v>13</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>11302</v>
+        <v>11303</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>2018</v>

</xml_diff>